<commit_message>
Preenche os 22 vídeos sem áudio no podcast com a análise do NotebookLM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0193kkcaFr2zeWvcQdmPTqWt
</commit_message>
<xml_diff>
--- a/sermoes/sermoes_fdqc_preenchida.xlsx
+++ b/sermoes/sermoes_fdqc_preenchida.xlsx
@@ -10351,15 +10351,25 @@
           <t>~2019</t>
         </is>
       </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Rt 1–4</t>
+        </is>
+      </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Sem áudio próprio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J165" s="4" t="n"/>
       <c r="L165" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=jFc2sOuPvys</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>Rute 1:1-21; 2:5-12; 3:9-12; 4:6-18</t>
         </is>
       </c>
     </row>
@@ -11208,15 +11218,25 @@
           <t>~2018</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Ef 1.1-14</t>
+        </is>
+      </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J179" s="4" t="n"/>
       <c r="L179" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=qXL1mkpAtu4</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Efésios 1:1-14; Efésios 2:10, 22; Ezequiel 36:25-28</t>
         </is>
       </c>
     </row>
@@ -11249,15 +11269,25 @@
           <t>~2018</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>1Co 11.17-34; Rm 12</t>
+        </is>
+      </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J180" s="4" t="n"/>
       <c r="L180" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=z_MSUPJTuNU</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>1 Coríntios 11:17-34; Romanos 12:1-21 (resposta quase idêntica à de "Para que nos reunimos?" — conferir)</t>
         </is>
       </c>
     </row>
@@ -11290,15 +11320,25 @@
           <t>~2018</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Mt 16.13-19</t>
+        </is>
+      </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J181" s="4" t="n"/>
       <c r="L181" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=9Lc8RamwSfY</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>Mateus 16:13-19; 1 Timóteo 3:15; Efésios 3:9-10; Atos 20:24; Lucas 4:43; Apocalipse 14:6; Números 16:41-50</t>
         </is>
       </c>
     </row>
@@ -11331,15 +11371,25 @@
           <t>~2018</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Ef 4.1-16</t>
+        </is>
+      </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J182" s="4" t="n"/>
       <c r="L182" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=URLxnlIMpvc</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>Efésios 4:1-16; Efésios 1:18; 3:18-19; 2 Pedro 1:3-11</t>
         </is>
       </c>
     </row>
@@ -11372,15 +11422,25 @@
           <t>~2018</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Ap 3.1-3</t>
+        </is>
+      </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J183" s="4" t="n"/>
       <c r="L183" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=y5RaaLVs4FY</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Apocalipse 3:1-3; Gênesis 6:9; Mateus 24:38; 1 Tessalonicenses 5:3; 2 Coríntios 5:17-20</t>
         </is>
       </c>
     </row>
@@ -11413,15 +11473,25 @@
           <t>~2018</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Gn 4.17-24; Jr 29.4-7</t>
+        </is>
+      </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J184" s="4" t="n"/>
       <c r="L184" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=37Ctc3FJ46k</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Gênesis 4:17-24; Mateus 9:35-38; Jeremias 29:4-7; Hebreus 11:8-10</t>
         </is>
       </c>
     </row>
@@ -11454,15 +11524,25 @@
           <t>~2018</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>1Co 11.17-34; Rm 12.1-2</t>
+        </is>
+      </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J185" s="4" t="n"/>
       <c r="L185" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=T_Df7pxWru4</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>1 Coríntios 11:17-34; Romanos 12:1-2</t>
         </is>
       </c>
     </row>
@@ -11490,15 +11570,25 @@
           <t>~dez/2025</t>
         </is>
       </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Lc 2.8-20</t>
+        </is>
+      </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J186" s="4" t="n"/>
       <c r="L186" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=LVp1npjJ7Qk</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Lucas 2:8-20; Gênesis 3:15; Isaías 9:2-6; Jeremias 29:13</t>
         </is>
       </c>
     </row>
@@ -11526,15 +11616,25 @@
           <t>~2024</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Is 7.14; Mt 1.23; Is 53</t>
+        </is>
+      </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Temático / vários textos</t>
         </is>
       </c>
       <c r="J187" s="4" t="n"/>
       <c r="L187" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=G2Ggf1Mr4TI</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Isaías 7:14 / Mateus 1:23; Isaías 53; panorama da história da redenção (cantata)</t>
         </is>
       </c>
     </row>
@@ -11567,15 +11667,25 @@
           <t>~dez/2024</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Is 9.6</t>
+        </is>
+      </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J188" s="4" t="n"/>
       <c r="L188" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Te5QQIv4vuA</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>Isaías 9:6</t>
         </is>
       </c>
     </row>
@@ -11603,15 +11713,25 @@
           <t>~dez/2023</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Jo 1.1-3; Mt 1.21; Ap 21.1-4 (vários textos)</t>
+        </is>
+      </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Temático / vários textos</t>
         </is>
       </c>
       <c r="J189" s="4" t="n"/>
       <c r="L189" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=rnyN95QCvDg</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>João 1:1-3; 2 Timóteo 1:8-10; Romanos 3:23; Mateus 1:21; 2:1-2; Tito 2:11-13; Apocalipse 21:1-4</t>
         </is>
       </c>
     </row>
@@ -11644,15 +11764,25 @@
           <t>~2023</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Mt 1.18-23; Lc 1.26-38</t>
+        </is>
+      </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J190" s="4" t="n"/>
       <c r="L190" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=rpUmvWkIKsw</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>Mateus 1:1-17; 1:18-23; Lucas 1:26-38; 2:10-14</t>
         </is>
       </c>
     </row>
@@ -12090,15 +12220,25 @@
           <t>Datas especiais e sermões avulsos</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>1Co 15.21-28</t>
+        </is>
+      </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J198" s="4" t="n"/>
       <c r="L198" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=-roaRFAQ0zM</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>1 Coríntios 15:21-28; 1 Coríntios 11; Romanos 3:23</t>
         </is>
       </c>
     </row>
@@ -12552,15 +12692,25 @@
           <t>~2019-2020</t>
         </is>
       </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Sl 89</t>
+        </is>
+      </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Provável — revisar</t>
         </is>
       </c>
       <c r="J206" s="4" t="n"/>
       <c r="L206" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=f-66VyYLImk</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>Salmo 89:1-52; Isaías 26:9; Salmos 73 e 74; Jeremias 29:11</t>
         </is>
       </c>
     </row>
@@ -12593,15 +12743,25 @@
           <t>~2019-2020</t>
         </is>
       </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Is 26.9; Am 3.6; Rm 5.8-9 (vários textos)</t>
+        </is>
+      </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Temático / vários textos</t>
         </is>
       </c>
       <c r="J207" s="4" t="n"/>
       <c r="L207" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=kpqtWTruD-0</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Isaías 26:9; Amós 3:6; Romanos 3:23; 5:8-9; 1 Coríntios 15:19</t>
         </is>
       </c>
     </row>
@@ -12634,15 +12794,25 @@
           <t>~2019-2020</t>
         </is>
       </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>2Tm 1.7; Mt 24.6; Mt 13 (vários textos)</t>
+        </is>
+      </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Temático / vários textos</t>
         </is>
       </c>
       <c r="J208" s="4" t="n"/>
       <c r="L208" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=yMJ11VbkhRU</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>2 Timóteo 1:7; Mateus 24:6; Mateus 13; Tito 2:13; 2 Pedro 3:12</t>
         </is>
       </c>
     </row>
@@ -13000,15 +13170,25 @@
           <t>Pregadores convidados, conferências e outros conteúdos</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Sl 96.1-13</t>
+        </is>
+      </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Não se aplica (palestra/podcast)</t>
         </is>
       </c>
       <c r="J215" s="4" t="n"/>
       <c r="L215" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=FHPHIvSrL9M</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>Salmo 96:1-13 (paralelo: 1 Crônicas 16:23-33)</t>
         </is>
       </c>
     </row>
@@ -13038,13 +13218,18 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Não se aplica (palestra/podcast)</t>
         </is>
       </c>
       <c r="J216" s="4" t="n"/>
       <c r="L216" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=GaPoGvwFUr0</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Painel de perguntas e respostas (sem texto base)</t>
         </is>
       </c>
     </row>
@@ -13072,15 +13257,25 @@
           <t>~2024</t>
         </is>
       </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>2Ts 2.1-4; Hb 11.13-16</t>
+        </is>
+      </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Não se aplica (palestra/podcast)</t>
         </is>
       </c>
       <c r="J217" s="4" t="n"/>
       <c r="L217" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=eLvum_z7Z_4</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>2 Tessalonicenses 2:1-4; 1 Pedro; Hebreus 11:13-16</t>
         </is>
       </c>
     </row>
@@ -13108,15 +13303,25 @@
           <t>~2024</t>
         </is>
       </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Rm 1.18-25; 12.2</t>
+        </is>
+      </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Não se aplica (palestra/podcast)</t>
         </is>
       </c>
       <c r="J218" s="4" t="n"/>
       <c r="L218" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=q-GHhd4dO7E</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Romanos 1:18-25; Romanos 12:2</t>
         </is>
       </c>
     </row>
@@ -13146,13 +13351,18 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>Sem áudio no podcast — usar NotebookLM</t>
+          <t>Não se aplica (palestra/podcast)</t>
         </is>
       </c>
       <c r="J219" s="4" t="n"/>
       <c r="L219" s="4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=fc8qbdZEx1g</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Palestra temática (sem texto base)</t>
         </is>
       </c>
     </row>
@@ -14771,7 +14981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -14784,7 +14994,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -14831,6 +15040,13 @@
       <c r="A9" t="inlineStr">
         <is>
           <t>• Linhas sem áudio no podcast: usar o NotebookLM com o link do YouTube (prompt no README).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>• Coluna "NotebookLM": resposta do NotebookLM. Para os 22 vídeos sem áudio no podcast, ele é a única fonte, por isso o status é no máximo "Provável".</t>
         </is>
       </c>
     </row>

</xml_diff>